<commit_message>
fix(lib): missing score definition on cyfun 2025 (#2741)
</commit_message>
<xml_diff>
--- a/tools/excel/ccb/cyfun2025.xlsx
+++ b/tools/excel/ccb/cyfun2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11003"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ericlaubacher/Documents/GitHub/ciso-assistant-community/tools/excel/ccb/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abder/mydev/intuitem/staging/ciso-assistant-community/tools/excel/ccb/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09C77A99-4EB4-584B-A9DE-FE29AA3BC953}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA9AE6B8-4C7B-2044-8556-59D83B060D4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28800" yWindow="-28180" windowWidth="51200" windowHeight="26920" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25680" yWindow="-28020" windowWidth="25360" windowHeight="27860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="2" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1433" uniqueCount="981">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1439" uniqueCount="986">
   <si>
     <t>GV.OC-01.1</t>
   </si>
@@ -5719,6 +5719,21 @@
 · Training and Drills: Conduct regular training sessions and crisis simulations to ensure the team is prepared to respond effectively.
 · Monitor and Adapt: Continuously monitor the situation and adapt the communication strategy as needed to address evolving circumstances.
 · Post-Crisis Review: After the crisis, review the communication efforts to identify lessons learned and improve future responses.</t>
+  </si>
+  <si>
+    <t>min_score</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>max_score</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>scores_definition</t>
   </si>
 </sst>
 </file>
@@ -5960,7 +5975,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -5971,7 +5986,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -5990,10 +6005,10 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -6053,10 +6068,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -6140,9 +6152,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -6156,13 +6165,13 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6497,7 +6506,7 @@
         <v>195</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -6570,7 +6579,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04BAF61A-04DC-E843-B98B-FBB8A932C760}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="28.33203125" bestFit="1" customWidth="1"/>
@@ -6631,6 +6640,30 @@
       </c>
       <c r="B7" t="s">
         <v>213</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>981</v>
+      </c>
+      <c r="B8" t="s">
+        <v>982</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>983</v>
+      </c>
+      <c r="B9" t="s">
+        <v>984</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>985</v>
+      </c>
+      <c r="B10" t="s">
+        <v>234</v>
       </c>
     </row>
   </sheetData>
@@ -8817,7 +8850,7 @@
       <c r="D126" t="s">
         <v>256</v>
       </c>
-      <c r="F126" s="35" t="s">
+      <c r="F126" s="34" t="s">
         <v>407</v>
       </c>
       <c r="G126" s="2" t="s">
@@ -8975,7 +9008,7 @@
       <c r="D136" t="s">
         <v>249</v>
       </c>
-      <c r="F136" s="37" t="s">
+      <c r="F136" s="36" t="s">
         <v>428</v>
       </c>
       <c r="G136" s="2" t="s">
@@ -8995,7 +9028,7 @@
       <c r="D137" t="s">
         <v>249</v>
       </c>
-      <c r="F137" s="36" t="s">
+      <c r="F137" s="35" t="s">
         <v>430</v>
       </c>
       <c r="G137" s="2" t="s">
@@ -9015,7 +9048,7 @@
       <c r="D138" t="s">
         <v>259</v>
       </c>
-      <c r="F138" s="36" t="s">
+      <c r="F138" s="35" t="s">
         <v>432</v>
       </c>
       <c r="G138" s="2" t="s">
@@ -9035,7 +9068,7 @@
       <c r="D139" t="s">
         <v>249</v>
       </c>
-      <c r="F139" s="36" t="s">
+      <c r="F139" s="35" t="s">
         <v>434</v>
       </c>
       <c r="G139" s="2" t="s">
@@ -9055,7 +9088,7 @@
       <c r="D140" t="s">
         <v>249</v>
       </c>
-      <c r="F140" s="36" t="s">
+      <c r="F140" s="35" t="s">
         <v>436</v>
       </c>
       <c r="G140" s="2" t="s">
@@ -9075,7 +9108,7 @@
       <c r="D141" t="s">
         <v>249</v>
       </c>
-      <c r="F141" s="36" t="s">
+      <c r="F141" s="35" t="s">
         <v>439</v>
       </c>
       <c r="G141" s="2" t="s">
@@ -9149,7 +9182,7 @@
       <c r="C145" t="s">
         <v>442</v>
       </c>
-      <c r="F145" s="36" t="s">
+      <c r="F145" s="35" t="s">
         <v>462</v>
       </c>
     </row>
@@ -9166,7 +9199,7 @@
       <c r="D146" t="s">
         <v>259</v>
       </c>
-      <c r="F146" s="36" t="s">
+      <c r="F146" s="35" t="s">
         <v>440</v>
       </c>
       <c r="G146" s="2" t="s">
@@ -9356,7 +9389,7 @@
       <c r="D157" t="s">
         <v>249</v>
       </c>
-      <c r="F157" s="38" t="s">
+      <c r="F157" s="37" t="s">
         <v>481</v>
       </c>
       <c r="G157" s="2" t="s">
@@ -9376,7 +9409,7 @@
       <c r="D158" t="s">
         <v>239</v>
       </c>
-      <c r="F158" s="39" t="s">
+      <c r="F158" s="38" t="s">
         <v>624</v>
       </c>
       <c r="G158" s="2" t="s">
@@ -9390,7 +9423,7 @@
       <c r="C159" t="s">
         <v>584</v>
       </c>
-      <c r="F159" s="39" t="s">
+      <c r="F159" s="38" t="s">
         <v>597</v>
       </c>
     </row>
@@ -9407,7 +9440,7 @@
       <c r="D160" t="s">
         <v>250</v>
       </c>
-      <c r="F160" s="39" t="s">
+      <c r="F160" s="38" t="s">
         <v>483</v>
       </c>
       <c r="G160" s="2" t="s">
@@ -9427,7 +9460,7 @@
       <c r="D161" t="s">
         <v>322</v>
       </c>
-      <c r="F161" s="40" t="s">
+      <c r="F161" s="39" t="s">
         <v>487</v>
       </c>
       <c r="G161" s="2" t="s">
@@ -9447,7 +9480,7 @@
       <c r="D162" t="s">
         <v>582</v>
       </c>
-      <c r="F162" s="41" t="s">
+      <c r="F162" s="40" t="s">
         <v>488</v>
       </c>
       <c r="G162" s="2" t="s">
@@ -9467,7 +9500,7 @@
       <c r="D163" t="s">
         <v>239</v>
       </c>
-      <c r="F163" s="63" t="s">
+      <c r="F163" s="35" t="s">
         <v>631</v>
       </c>
       <c r="G163" s="2" t="s">
@@ -9487,7 +9520,7 @@
       <c r="D164" t="s">
         <v>239</v>
       </c>
-      <c r="F164" s="63" t="s">
+      <c r="F164" s="35" t="s">
         <v>632</v>
       </c>
       <c r="G164" s="2" t="s">
@@ -9501,7 +9534,7 @@
       <c r="C165" t="s">
         <v>635</v>
       </c>
-      <c r="F165" s="63" t="s">
+      <c r="F165" s="35" t="s">
         <v>634</v>
       </c>
     </row>
@@ -9518,7 +9551,7 @@
       <c r="D166" t="s">
         <v>239</v>
       </c>
-      <c r="F166" s="63" t="s">
+      <c r="F166" s="35" t="s">
         <v>634</v>
       </c>
       <c r="G166" s="2" t="s">
@@ -9532,7 +9565,7 @@
       <c r="C167" t="s">
         <v>583</v>
       </c>
-      <c r="F167" s="63" t="s">
+      <c r="F167" s="35" t="s">
         <v>598</v>
       </c>
     </row>
@@ -9549,7 +9582,7 @@
       <c r="D168" t="s">
         <v>322</v>
       </c>
-      <c r="F168" s="42" t="s">
+      <c r="F168" s="41" t="s">
         <v>489</v>
       </c>
       <c r="G168" s="2" t="s">
@@ -9569,7 +9602,7 @@
       <c r="D169" t="s">
         <v>322</v>
       </c>
-      <c r="F169" s="40" t="s">
+      <c r="F169" s="39" t="s">
         <v>491</v>
       </c>
       <c r="G169" s="2" t="s">
@@ -9589,7 +9622,7 @@
       <c r="D170" t="s">
         <v>322</v>
       </c>
-      <c r="F170" s="43" t="s">
+      <c r="F170" s="42" t="s">
         <v>498</v>
       </c>
       <c r="G170" s="2" t="s">
@@ -9609,7 +9642,7 @@
       <c r="D171" t="s">
         <v>322</v>
       </c>
-      <c r="F171" s="41" t="s">
+      <c r="F171" s="40" t="s">
         <v>499</v>
       </c>
       <c r="G171" s="2" t="s">
@@ -9629,7 +9662,7 @@
       <c r="D172" t="s">
         <v>249</v>
       </c>
-      <c r="F172" s="37" t="s">
+      <c r="F172" s="36" t="s">
         <v>500</v>
       </c>
       <c r="G172" s="2" t="s">
@@ -9669,7 +9702,7 @@
       <c r="D174" t="s">
         <v>249</v>
       </c>
-      <c r="F174" s="44" t="s">
+      <c r="F174" s="43" t="s">
         <v>502</v>
       </c>
       <c r="G174" s="2" t="s">
@@ -9689,7 +9722,7 @@
       <c r="D175" t="s">
         <v>239</v>
       </c>
-      <c r="F175" s="61" t="s">
+      <c r="F175" s="60" t="s">
         <v>646</v>
       </c>
       <c r="G175" s="2" t="s">
@@ -9709,7 +9742,7 @@
       <c r="D176" t="s">
         <v>239</v>
       </c>
-      <c r="F176" s="61" t="s">
+      <c r="F176" s="60" t="s">
         <v>649</v>
       </c>
       <c r="G176" s="2" t="s">
@@ -9723,7 +9756,7 @@
       <c r="C177" t="s">
         <v>585</v>
       </c>
-      <c r="F177" s="61" t="s">
+      <c r="F177" s="60" t="s">
         <v>599</v>
       </c>
     </row>
@@ -9760,7 +9793,7 @@
       <c r="D179" t="s">
         <v>249</v>
       </c>
-      <c r="F179" s="45" t="s">
+      <c r="F179" s="44" t="s">
         <v>506</v>
       </c>
       <c r="G179" s="2" t="s">
@@ -9780,7 +9813,7 @@
       <c r="D180" t="s">
         <v>239</v>
       </c>
-      <c r="F180" s="62" t="s">
+      <c r="F180" s="61" t="s">
         <v>655</v>
       </c>
       <c r="G180" s="2" t="s">
@@ -9800,7 +9833,7 @@
       <c r="D181" t="s">
         <v>239</v>
       </c>
-      <c r="F181" s="62" t="s">
+      <c r="F181" s="61" t="s">
         <v>657</v>
       </c>
       <c r="G181" s="2" t="s">
@@ -9817,7 +9850,7 @@
       <c r="E182" s="5" t="s">
         <v>590</v>
       </c>
-      <c r="F182" s="62" t="s">
+      <c r="F182" s="61" t="s">
         <v>592</v>
       </c>
     </row>
@@ -9828,7 +9861,7 @@
       <c r="C183" t="s">
         <v>566</v>
       </c>
-      <c r="F183" s="62" t="s">
+      <c r="F183" s="61" t="s">
         <v>600</v>
       </c>
     </row>
@@ -9845,7 +9878,7 @@
       <c r="D184" t="s">
         <v>250</v>
       </c>
-      <c r="F184" s="46" t="s">
+      <c r="F184" s="45" t="s">
         <v>507</v>
       </c>
       <c r="G184" s="2" t="s">
@@ -9865,7 +9898,7 @@
       <c r="D185" t="s">
         <v>249</v>
       </c>
-      <c r="F185" s="58" t="s">
+      <c r="F185" s="57" t="s">
         <v>512</v>
       </c>
       <c r="G185" s="2" t="s">
@@ -9885,7 +9918,7 @@
       <c r="D186" t="s">
         <v>249</v>
       </c>
-      <c r="F186" s="57" t="s">
+      <c r="F186" s="56" t="s">
         <v>511</v>
       </c>
       <c r="G186" s="2" t="s">
@@ -9993,7 +10026,7 @@
       <c r="E192" s="5" t="s">
         <v>589</v>
       </c>
-      <c r="F192" s="36" t="s">
+      <c r="F192" s="35" t="s">
         <v>591</v>
       </c>
     </row>
@@ -10004,7 +10037,7 @@
       <c r="C193" t="s">
         <v>568</v>
       </c>
-      <c r="F193" s="36" t="s">
+      <c r="F193" s="35" t="s">
         <v>602</v>
       </c>
     </row>
@@ -10021,7 +10054,7 @@
       <c r="D194" t="s">
         <v>249</v>
       </c>
-      <c r="F194" s="47" t="s">
+      <c r="F194" s="46" t="s">
         <v>519</v>
       </c>
       <c r="G194" s="2" t="s">
@@ -10121,7 +10154,7 @@
       <c r="D199" t="s">
         <v>239</v>
       </c>
-      <c r="F199" s="64" t="s">
+      <c r="F199" s="62" t="s">
         <v>678</v>
       </c>
       <c r="G199" s="2" t="s">
@@ -10141,7 +10174,7 @@
       <c r="D200" t="s">
         <v>250</v>
       </c>
-      <c r="F200" s="48" t="s">
+      <c r="F200" s="47" t="s">
         <v>525</v>
       </c>
       <c r="G200" s="2" t="s">
@@ -10155,7 +10188,7 @@
       <c r="C201" t="s">
         <v>681</v>
       </c>
-      <c r="F201" s="36" t="s">
+      <c r="F201" s="35" t="s">
         <v>682</v>
       </c>
     </row>
@@ -10172,7 +10205,7 @@
       <c r="D202" t="s">
         <v>258</v>
       </c>
-      <c r="F202" s="36" t="s">
+      <c r="F202" s="35" t="s">
         <v>684</v>
       </c>
       <c r="G202" s="2" t="s">
@@ -10192,7 +10225,7 @@
       <c r="D203" t="s">
         <v>239</v>
       </c>
-      <c r="F203" s="36" t="s">
+      <c r="F203" s="35" t="s">
         <v>686</v>
       </c>
       <c r="G203" s="2" t="s">
@@ -10206,7 +10239,7 @@
       <c r="C204" t="s">
         <v>689</v>
       </c>
-      <c r="F204" s="36" t="s">
+      <c r="F204" s="35" t="s">
         <v>690</v>
       </c>
       <c r="G204" s="2"/>
@@ -10224,7 +10257,7 @@
       <c r="D205" t="s">
         <v>239</v>
       </c>
-      <c r="F205" s="36" t="s">
+      <c r="F205" s="35" t="s">
         <v>692</v>
       </c>
       <c r="G205" s="2" t="s">
@@ -10238,7 +10271,7 @@
       <c r="C206" t="s">
         <v>569</v>
       </c>
-      <c r="F206" s="36" t="s">
+      <c r="F206" s="35" t="s">
         <v>603</v>
       </c>
     </row>
@@ -10255,7 +10288,7 @@
       <c r="D207" t="s">
         <v>322</v>
       </c>
-      <c r="F207" s="49" t="s">
+      <c r="F207" s="48" t="s">
         <v>527</v>
       </c>
       <c r="G207" s="2" t="s">
@@ -10275,7 +10308,7 @@
       <c r="D208" t="s">
         <v>249</v>
       </c>
-      <c r="F208" s="50" t="s">
+      <c r="F208" s="49" t="s">
         <v>531</v>
       </c>
       <c r="G208" s="2" t="s">
@@ -10295,7 +10328,7 @@
       <c r="D209" t="s">
         <v>249</v>
       </c>
-      <c r="F209" s="51" t="s">
+      <c r="F209" s="50" t="s">
         <v>532</v>
       </c>
       <c r="G209" s="2" t="s">
@@ -10315,7 +10348,7 @@
       <c r="D210" t="s">
         <v>239</v>
       </c>
-      <c r="F210" s="54" t="s">
+      <c r="F210" s="53" t="s">
         <v>698</v>
       </c>
       <c r="G210" s="2" t="s">
@@ -10335,7 +10368,7 @@
       <c r="D211" t="s">
         <v>239</v>
       </c>
-      <c r="F211" s="54" t="s">
+      <c r="F211" s="53" t="s">
         <v>701</v>
       </c>
       <c r="G211" s="2" t="s">
@@ -10352,7 +10385,7 @@
       <c r="E212" s="5" t="s">
         <v>595</v>
       </c>
-      <c r="F212" s="54" t="s">
+      <c r="F212" s="53" t="s">
         <v>594</v>
       </c>
     </row>
@@ -10363,7 +10396,7 @@
       <c r="C213" t="s">
         <v>570</v>
       </c>
-      <c r="F213" s="54" t="s">
+      <c r="F213" s="53" t="s">
         <v>604</v>
       </c>
     </row>
@@ -10400,7 +10433,7 @@
       <c r="D215" t="s">
         <v>239</v>
       </c>
-      <c r="F215" s="63" t="s">
+      <c r="F215" s="35" t="s">
         <v>708</v>
       </c>
       <c r="G215" s="2" t="s">
@@ -10474,7 +10507,7 @@
       <c r="C219" t="s">
         <v>573</v>
       </c>
-      <c r="F219" s="63" t="s">
+      <c r="F219" s="35" t="s">
         <v>605</v>
       </c>
     </row>
@@ -10491,7 +10524,7 @@
       <c r="D220" t="s">
         <v>249</v>
       </c>
-      <c r="F220" s="52" t="s">
+      <c r="F220" s="51" t="s">
         <v>535</v>
       </c>
       <c r="G220" s="2" t="s">
@@ -10505,7 +10538,7 @@
       <c r="C221" t="s">
         <v>574</v>
       </c>
-      <c r="F221" s="52" t="s">
+      <c r="F221" s="51" t="s">
         <v>606</v>
       </c>
     </row>
@@ -10522,7 +10555,7 @@
       <c r="D222" t="s">
         <v>249</v>
       </c>
-      <c r="F222" s="52" t="s">
+      <c r="F222" s="51" t="s">
         <v>537</v>
       </c>
       <c r="G222" s="2" t="s">
@@ -10536,7 +10569,7 @@
       <c r="C223" t="s">
         <v>575</v>
       </c>
-      <c r="F223" s="55" t="s">
+      <c r="F223" s="54" t="s">
         <v>607</v>
       </c>
     </row>
@@ -10553,7 +10586,7 @@
       <c r="D224" t="s">
         <v>322</v>
       </c>
-      <c r="F224" s="59" t="s">
+      <c r="F224" s="58" t="s">
         <v>539</v>
       </c>
       <c r="G224" s="2" t="s">
@@ -10573,7 +10606,7 @@
       <c r="D225" t="s">
         <v>249</v>
       </c>
-      <c r="F225" s="53" t="s">
+      <c r="F225" s="52" t="s">
         <v>544</v>
       </c>
       <c r="G225" s="2" t="s">
@@ -10593,7 +10626,7 @@
       <c r="D226" t="s">
         <v>249</v>
       </c>
-      <c r="F226" s="54" t="s">
+      <c r="F226" s="53" t="s">
         <v>543</v>
       </c>
       <c r="G226" s="2" t="s">
@@ -10647,7 +10680,7 @@
       <c r="C229" t="s">
         <v>576</v>
       </c>
-      <c r="F229" s="50" t="s">
+      <c r="F229" s="49" t="s">
         <v>608</v>
       </c>
     </row>
@@ -10664,7 +10697,7 @@
       <c r="D230" t="s">
         <v>250</v>
       </c>
-      <c r="F230" s="55" t="s">
+      <c r="F230" s="54" t="s">
         <v>545</v>
       </c>
       <c r="G230" s="2" t="s">
@@ -10684,7 +10717,7 @@
       <c r="D231" t="s">
         <v>249</v>
       </c>
-      <c r="F231" s="51" t="s">
+      <c r="F231" s="50" t="s">
         <v>548</v>
       </c>
       <c r="G231" s="2" t="s">
@@ -10698,7 +10731,7 @@
       <c r="C232" t="s">
         <v>577</v>
       </c>
-      <c r="F232" s="50" t="s">
+      <c r="F232" s="49" t="s">
         <v>609</v>
       </c>
     </row>
@@ -10715,7 +10748,7 @@
       <c r="D233" t="s">
         <v>249</v>
       </c>
-      <c r="F233" s="55" t="s">
+      <c r="F233" s="54" t="s">
         <v>549</v>
       </c>
       <c r="G233" s="2" t="s">
@@ -10735,7 +10768,7 @@
       <c r="D234" t="s">
         <v>249</v>
       </c>
-      <c r="F234" s="51" t="s">
+      <c r="F234" s="50" t="s">
         <v>551</v>
       </c>
       <c r="G234" s="2" t="s">
@@ -10755,7 +10788,7 @@
       <c r="D235" t="s">
         <v>239</v>
       </c>
-      <c r="F235" s="50" t="s">
+      <c r="F235" s="49" t="s">
         <v>733</v>
       </c>
       <c r="G235" s="2" t="s">
@@ -10792,7 +10825,7 @@
       <c r="E237" s="5" t="s">
         <v>588</v>
       </c>
-      <c r="F237" s="50" t="s">
+      <c r="F237" s="49" t="s">
         <v>587</v>
       </c>
     </row>
@@ -10803,7 +10836,7 @@
       <c r="C238" t="s">
         <v>578</v>
       </c>
-      <c r="F238" s="50" t="s">
+      <c r="F238" s="49" t="s">
         <v>610</v>
       </c>
     </row>
@@ -10820,7 +10853,7 @@
       <c r="D239" t="s">
         <v>322</v>
       </c>
-      <c r="F239" s="49" t="s">
+      <c r="F239" s="48" t="s">
         <v>553</v>
       </c>
       <c r="G239" s="2" t="s">
@@ -10840,7 +10873,7 @@
       <c r="D240" t="s">
         <v>322</v>
       </c>
-      <c r="F240" s="56" t="s">
+      <c r="F240" s="55" t="s">
         <v>555</v>
       </c>
       <c r="G240" s="2" t="s">
@@ -10860,7 +10893,7 @@
       <c r="D241" t="s">
         <v>582</v>
       </c>
-      <c r="F241" s="40" t="s">
+      <c r="F241" s="39" t="s">
         <v>559</v>
       </c>
       <c r="G241" s="2" t="s">
@@ -10880,7 +10913,7 @@
       <c r="D242" t="s">
         <v>582</v>
       </c>
-      <c r="F242" s="41" t="s">
+      <c r="F242" s="40" t="s">
         <v>560</v>
       </c>
       <c r="G242" s="2" t="s">
@@ -10994,7 +11027,7 @@
       <c r="C248" t="s">
         <v>580</v>
       </c>
-      <c r="F248" s="63" t="s">
+      <c r="F248" s="35" t="s">
         <v>611</v>
       </c>
     </row>
@@ -11011,7 +11044,7 @@
       <c r="D249" t="s">
         <v>249</v>
       </c>
-      <c r="F249" s="52" t="s">
+      <c r="F249" s="51" t="s">
         <v>561</v>
       </c>
       <c r="G249" s="2" t="s">
@@ -11031,7 +11064,7 @@
       <c r="D250" t="s">
         <v>239</v>
       </c>
-      <c r="F250" s="52" t="s">
+      <c r="F250" s="51" t="s">
         <v>758</v>
       </c>
       <c r="G250" s="2" t="s">
@@ -11045,7 +11078,7 @@
       <c r="C251" t="s">
         <v>760</v>
       </c>
-      <c r="F251" s="52" t="s">
+      <c r="F251" s="51" t="s">
         <v>765</v>
       </c>
       <c r="G251" s="2"/>
@@ -11077,7 +11110,7 @@
       <c r="C253" t="s">
         <v>581</v>
       </c>
-      <c r="F253" s="52" t="s">
+      <c r="F253" s="51" t="s">
         <v>612</v>
       </c>
     </row>
@@ -11094,7 +11127,7 @@
       <c r="D254" t="s">
         <v>249</v>
       </c>
-      <c r="F254" s="52" t="s">
+      <c r="F254" s="51" t="s">
         <v>563</v>
       </c>
       <c r="G254" s="2" t="s">
@@ -11136,7 +11169,7 @@
         <v>770</v>
       </c>
       <c r="E257" s="2"/>
-      <c r="F257" s="34" t="s">
+      <c r="F257" s="2" t="s">
         <v>774</v>
       </c>
     </row>
@@ -11153,7 +11186,7 @@
       <c r="D258" t="s">
         <v>250</v>
       </c>
-      <c r="F258" s="39" t="s">
+      <c r="F258" s="38" t="s">
         <v>820</v>
       </c>
       <c r="G258" s="2" t="s">
@@ -11173,7 +11206,7 @@
       <c r="D259" t="s">
         <v>322</v>
       </c>
-      <c r="F259" s="65" t="s">
+      <c r="F259" s="63" t="s">
         <v>821</v>
       </c>
       <c r="G259" s="2" t="s">
@@ -11193,7 +11226,7 @@
       <c r="D260" t="s">
         <v>582</v>
       </c>
-      <c r="F260" s="60" t="s">
+      <c r="F260" s="59" t="s">
         <v>822</v>
       </c>
       <c r="G260" s="2" t="s">
@@ -11295,7 +11328,7 @@
       <c r="D266" t="s">
         <v>250</v>
       </c>
-      <c r="F266" s="39" t="s">
+      <c r="F266" s="38" t="s">
         <v>783</v>
       </c>
       <c r="G266" s="2" t="s">
@@ -11315,7 +11348,7 @@
       <c r="D267" t="s">
         <v>249</v>
       </c>
-      <c r="F267" s="66" t="s">
+      <c r="F267" s="64" t="s">
         <v>786</v>
       </c>
       <c r="G267" s="2" t="s">
@@ -11337,7 +11370,7 @@
       <c r="A269" t="s">
         <v>126</v>
       </c>
-      <c r="B269" s="68">
+      <c r="B269" s="66">
         <v>4</v>
       </c>
       <c r="C269" t="s">
@@ -11346,7 +11379,7 @@
       <c r="D269" t="s">
         <v>249</v>
       </c>
-      <c r="F269" s="37" t="s">
+      <c r="F269" s="36" t="s">
         <v>789</v>
       </c>
       <c r="G269" s="2" t="s">
@@ -11357,7 +11390,7 @@
       <c r="A270" t="s">
         <v>126</v>
       </c>
-      <c r="B270" s="68">
+      <c r="B270" s="66">
         <v>4</v>
       </c>
       <c r="C270" t="s">
@@ -11366,7 +11399,7 @@
       <c r="D270" t="s">
         <v>249</v>
       </c>
-      <c r="F270" s="67" t="s">
+      <c r="F270" s="65" t="s">
         <v>792</v>
       </c>
       <c r="G270" s="2" t="s">
@@ -11553,7 +11586,7 @@
       <c r="D281" t="s">
         <v>322</v>
       </c>
-      <c r="F281" s="59" t="s">
+      <c r="F281" s="58" t="s">
         <v>806</v>
       </c>
       <c r="G281" s="2" t="s">
@@ -11573,7 +11606,7 @@
       <c r="D282" t="s">
         <v>249</v>
       </c>
-      <c r="F282" s="67" t="s">
+      <c r="F282" s="65" t="s">
         <v>809</v>
       </c>
       <c r="G282" s="2" t="s">
@@ -11607,7 +11640,7 @@
       <c r="C284" t="s">
         <v>817</v>
       </c>
-      <c r="F284" s="69" t="s">
+      <c r="F284" s="67" t="s">
         <v>818</v>
       </c>
     </row>
@@ -11624,7 +11657,7 @@
       <c r="D285" t="s">
         <v>256</v>
       </c>
-      <c r="F285" s="69" t="s">
+      <c r="F285" s="67" t="s">
         <v>858</v>
       </c>
       <c r="G285" s="2" t="s">
@@ -11744,7 +11777,7 @@
       <c r="D293" t="s">
         <v>250</v>
       </c>
-      <c r="F293" s="39" t="s">
+      <c r="F293" s="38" t="s">
         <v>868</v>
       </c>
       <c r="G293" s="2" t="s">
@@ -11764,7 +11797,7 @@
       <c r="D294" t="s">
         <v>249</v>
       </c>
-      <c r="F294" s="66" t="s">
+      <c r="F294" s="64" t="s">
         <v>871</v>
       </c>
       <c r="G294" s="2" t="s">
@@ -11795,7 +11828,7 @@
       <c r="D296" t="s">
         <v>249</v>
       </c>
-      <c r="F296" s="47" t="s">
+      <c r="F296" s="46" t="s">
         <v>874</v>
       </c>
       <c r="G296" s="2" t="s">
@@ -11815,7 +11848,7 @@
       <c r="D297" t="s">
         <v>239</v>
       </c>
-      <c r="F297" s="39" t="s">
+      <c r="F297" s="38" t="s">
         <v>904</v>
       </c>
       <c r="G297" s="2" t="s">
@@ -11829,7 +11862,7 @@
       <c r="C298" t="s">
         <v>877</v>
       </c>
-      <c r="F298" s="39" t="s">
+      <c r="F298" s="38" t="s">
         <v>876</v>
       </c>
     </row>
@@ -11846,7 +11879,7 @@
       <c r="D299" t="s">
         <v>249</v>
       </c>
-      <c r="F299" s="38" t="s">
+      <c r="F299" s="37" t="s">
         <v>907</v>
       </c>
       <c r="G299" s="2" t="s">
@@ -11860,7 +11893,7 @@
       <c r="C300" t="s">
         <v>880</v>
       </c>
-      <c r="F300" s="38" t="s">
+      <c r="F300" s="37" t="s">
         <v>879</v>
       </c>
     </row>
@@ -11877,7 +11910,7 @@
       <c r="D301" t="s">
         <v>249</v>
       </c>
-      <c r="F301" s="38" t="s">
+      <c r="F301" s="37" t="s">
         <v>881</v>
       </c>
       <c r="G301" s="2" t="s">
@@ -11891,7 +11924,7 @@
       <c r="C302" t="s">
         <v>910</v>
       </c>
-      <c r="E302" s="71" t="s">
+      <c r="E302" s="69" t="s">
         <v>911</v>
       </c>
       <c r="F302" s="2" t="s">
@@ -11906,7 +11939,7 @@
       <c r="C303" t="s">
         <v>914</v>
       </c>
-      <c r="E303" s="71"/>
+      <c r="E303" s="69"/>
       <c r="F303" s="2" t="s">
         <v>913</v>
       </c>
@@ -11925,7 +11958,7 @@
       <c r="D304" t="s">
         <v>239</v>
       </c>
-      <c r="E304" s="71"/>
+      <c r="E304" s="69"/>
       <c r="F304" s="2" t="s">
         <v>915</v>
       </c>
@@ -11940,7 +11973,7 @@
       <c r="C305" t="s">
         <v>918</v>
       </c>
-      <c r="E305" s="71"/>
+      <c r="E305" s="69"/>
       <c r="F305" s="2" t="s">
         <v>919</v>
       </c>
@@ -11959,7 +11992,7 @@
       <c r="D306" t="s">
         <v>239</v>
       </c>
-      <c r="E306" s="71"/>
+      <c r="E306" s="69"/>
       <c r="F306" s="2" t="s">
         <v>921</v>
       </c>
@@ -11974,7 +12007,7 @@
       <c r="C307" t="s">
         <v>923</v>
       </c>
-      <c r="E307" s="71"/>
+      <c r="E307" s="69"/>
       <c r="F307" s="2" t="s">
         <v>924</v>
       </c>
@@ -11993,7 +12026,7 @@
       <c r="D308" t="s">
         <v>239</v>
       </c>
-      <c r="E308" s="71"/>
+      <c r="E308" s="69"/>
       <c r="F308" s="2" t="s">
         <v>925</v>
       </c>
@@ -12008,7 +12041,7 @@
       <c r="C309" t="s">
         <v>929</v>
       </c>
-      <c r="E309" s="71"/>
+      <c r="E309" s="69"/>
       <c r="F309" s="2" t="s">
         <v>928</v>
       </c>
@@ -12027,7 +12060,7 @@
       <c r="D310" t="s">
         <v>239</v>
       </c>
-      <c r="E310" s="71"/>
+      <c r="E310" s="69"/>
       <c r="F310" s="2" t="s">
         <v>930</v>
       </c>
@@ -12073,7 +12106,7 @@
       <c r="D313" t="s">
         <v>250</v>
       </c>
-      <c r="F313" s="39" t="s">
+      <c r="F313" s="38" t="s">
         <v>888</v>
       </c>
       <c r="G313" s="2" t="s">
@@ -12093,7 +12126,7 @@
       <c r="D314" t="s">
         <v>582</v>
       </c>
-      <c r="F314" s="70" t="s">
+      <c r="F314" s="68" t="s">
         <v>891</v>
       </c>
       <c r="G314" s="2" t="s">
@@ -12138,7 +12171,7 @@
       <c r="D317" t="s">
         <v>249</v>
       </c>
-      <c r="F317" s="36" t="s">
+      <c r="F317" s="35" t="s">
         <v>897</v>
       </c>
       <c r="G317" s="2" t="s">
@@ -12158,7 +12191,7 @@
       <c r="D318" t="s">
         <v>582</v>
       </c>
-      <c r="F318" s="70" t="s">
+      <c r="F318" s="68" t="s">
         <v>900</v>
       </c>
       <c r="G318" s="2" t="s">

</xml_diff>

<commit_message>
fix(lib): missing ID.IM-03.1 item on basic level of Cyfun 2025 (#2796)
</commit_message>
<xml_diff>
--- a/tools/excel/ccb/cyfun2025.xlsx
+++ b/tools/excel/ccb/cyfun2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/abder/mydev/intuitem/staging/ciso-assistant-community/tools/excel/ccb/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA9AE6B8-4C7B-2044-8556-59D83B060D4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2082215A-E737-ED4D-BDFB-B1B64F818934}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25680" yWindow="-28020" windowWidth="25360" windowHeight="27860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4020" yWindow="-28020" windowWidth="50880" windowHeight="27860" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="2" r:id="rId1"/>
@@ -6506,7 +6506,7 @@
         <v>195</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -9006,7 +9006,7 @@
         <v>429</v>
       </c>
       <c r="D136" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F136" s="36" t="s">
         <v>428</v>

</xml_diff>

<commit_message>
[Excel] Fix Wrong/Missing Values
Changes :
Dans `requirements_content` :
L57 - `GV.SC-03.1`, `annotation[nl]`
L163 - `PR.AA-03.2`, `annotation[nl]`
L176 - `PR.AA-05.7`, `annotation[nl]`
L182 - `PR.AA-06.3`, `annotation[nl]`

Dans `controls_content` :
H30 - `GV.SC-03.1`, `annotation[nl]`
H105 - `PR.AA-03.2`, `annotation[nl]`
H116 - `PR.AA-05.7`, `annotation[nl]`
H121 - `PR.AA-06.3`, `annotation[nl]`
</commit_message>
<xml_diff>
--- a/tools/excel/ccb/cyfun2025.xlsx
+++ b/tools/excel/ccb/cyfun2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JulianDoloir\Desktop\Repos\intuitem\ciso-assistant-community\tools\excel\ccb\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3502BA9F-40EA-47AE-B126-D9618FF3D7FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7D9601C-E3E6-4FA3-9505-AEC925A2E7E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38064" yWindow="-10932" windowWidth="26400" windowHeight="17952" tabRatio="906" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25452" yWindow="-8148" windowWidth="26400" windowHeight="17952" tabRatio="906" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="1" r:id="rId1"/>
@@ -2380,6 +2380,9 @@
     -  Procesverbeteringscycli (bijv. PDCA)
 -  Beleid, procedures en controles bijwerken op basis van veranderende bedreigingen en leveranciersprestaties.
 Escaleren van materiële risico’s naar het senior management
+-  Definieer criteria voor materialiteit (bijv. financiële impact, blootstelling aan regelgeving, operationele verstoring).
+-  Zorg voor een formeel escalatiepad naar het senior management en risicocomités.
+-  Zorg ervoor dat materiële risico’s in de toeleveringsketen:
     -  worden weergegeven in het bedrijfsrisicoregister
     -  aan de orde komen in strategische risicodiscussies
     -  meegenomen worden in de planning voor bedrijfscontinuïteit en crisisbeheer</t>
@@ -6661,6 +6664,9 @@
     -  Er zou regelmatig opleiding kunnen worden gegeven om gebruikers bewust te maken van phishing.
 -  OT-specifieke overwegingen met betrekking tot MFA (zie ook PR.AA-01.1)
     -  Gedeelde toegang tot PLC’s/HMI’s
+-  Als individuele accounts niet haalbaar zijn, zou het principe van minimale rechten kunnen worden toegepast.
+        -  Er zou een beveiligde jumpserver of HMI-front-end kunnen worden gebruikt om de toegang te controleren, activiteiten te loggen en een authenticatielaag toe te voegen.
+    -  Veilige externe toegang tot OT-systemen
         -  De technische en procedurele vereisten voor toegang op afstand zouden duidelijk kunnen worden gedefinieerd.
         -  Er zouden veilige protocollen (bijv. VPN, SSH, TLS) kunnen worden gebruikt.
         -  MFA zou kunnen worden afgedwongen voor alle externe OT-toegang, met name voor externe leveranciers.
@@ -7473,7 +7479,10 @@
 -  Verdacht gedrag detecteren Afwijkend gedrag en ongeoorloofde acties zouden kunnen worden geïdentificeerd door middel van geautomatiseerde logboekregistratie en waarschuwingsmechanismen.
 -  Incidentrespons ondersteunen Monitoringgegevens zouden kunnen worden gebruikt om beveiligingsincidenten met geprivilegieerde accounts te onderzoeken en erop te reageren.
 -  Toegangsrechten proactief beheren Toegangsrechten zouden duidelijk kunnen worden gedefinieerd, regelmatig worden herzien en worden aangepast op basis van rolveranderingen, operationele behoeften of risicobeoordelingen.
--  Zorgen voor OT-specifieke haalbaarheid</t>
+-  Zorgen voor OT-specifieke haalbaarheid
+-  In OT-omgevingen zou geprivilegieerde toegang kunnen worden beheerd met inachtneming van de stabiliteit en veiligheid van het systeem.
+    -  Wanneer volledige monitoring niet haalbaar is, zouden compenserende controles zoals logging1 op interfaceniveau of externe beoordeling kunnen worden geïmplementeerd.
+-  Afstemmen op ENISA-richtlijnen Deze praktijken zouden in overeenstemming kunnen zijn met de technische implementatierichtlijnen van ENISA voor NIS2, waarin het belang van geprivilegieerde toegangscontrole en monitoring voor het beveiligen van essentiële diensten en kritieke infrastructuur wordt benadrukt.</t>
   </si>
   <si>
     <t>Les utilisateurs privilégiés doivent être gérés et surveillés.</t>
@@ -7880,6 +7889,7 @@
   <si>
     <t>Het doel van deze controle is het risico van ongeoorloofde fysieke toegang tot gebieden die essentieel zijn voor de bedrijfscontinuïteit, de integriteit van gegevens en de veiligheid van personeel en apparatuur te verminderen door strengere toegangsmaatregelen toe te passen dan die welke in algemene faciliteiten worden gebruikt.
 Om dit doel te bereiken, kan het volgende worden overwogen:
+-  Kritieke zones zouden geïdentificeerd kunnen worden tijdens de classificatie van assets. Deze omvatten doorgaans:
     -  Productie- en operationele technologie (OT)-omgevingen
     -  Serverruimtes en datacenters
     -  Financiële en personeelsafdelingen
@@ -20583,7 +20593,7 @@
       <c r="K57" s="13" t="s">
         <v>408</v>
       </c>
-      <c r="L57" s="13" t="s">
+      <c r="L57" s="62" t="s">
         <v>409</v>
       </c>
       <c r="M57" s="45"/>
@@ -24375,7 +24385,7 @@
       <c r="K163" s="4" t="s">
         <v>1149</v>
       </c>
-      <c r="L163" s="13" t="s">
+      <c r="L163" s="62" t="s">
         <v>1150</v>
       </c>
       <c r="M163" s="45"/>
@@ -24858,7 +24868,7 @@
       <c r="K176" s="29" t="s">
         <v>1242</v>
       </c>
-      <c r="L176" s="13" t="s">
+      <c r="L176" s="62" t="s">
         <v>1243</v>
       </c>
       <c r="M176" s="45"/>
@@ -25080,7 +25090,7 @@
       <c r="K182" s="31" t="s">
         <v>1286</v>
       </c>
-      <c r="L182" s="13" t="s">
+      <c r="L182" s="62" t="s">
         <v>1287</v>
       </c>
       <c r="M182" s="45"/>
@@ -25225,7 +25235,7 @@
       <c r="N186" s="34" t="s">
         <v>1315</v>
       </c>
-      <c r="O186" s="62" t="s">
+      <c r="O186" s="13" t="s">
         <v>1316</v>
       </c>
     </row>
@@ -26311,7 +26321,7 @@
       <c r="N216" s="4" t="s">
         <v>1529</v>
       </c>
-      <c r="O216" s="62" t="s">
+      <c r="O216" s="13" t="s">
         <v>1530</v>
       </c>
     </row>
@@ -31567,7 +31577,7 @@
       <c r="G30" s="13" t="s">
         <v>408</v>
       </c>
-      <c r="H30" s="14" t="s">
+      <c r="H30" s="63" t="s">
         <v>409</v>
       </c>
       <c r="I30" s="13" t="s">
@@ -34048,7 +34058,7 @@
       <c r="G105" s="4" t="s">
         <v>1149</v>
       </c>
-      <c r="H105" s="14" t="s">
+      <c r="H105" s="63" t="s">
         <v>1150</v>
       </c>
       <c r="I105" s="13" t="s">
@@ -34411,7 +34421,7 @@
       <c r="G116" s="29" t="s">
         <v>1242</v>
       </c>
-      <c r="H116" s="14" t="s">
+      <c r="H116" s="63" t="s">
         <v>1243</v>
       </c>
       <c r="I116" s="13" t="s">
@@ -34576,7 +34586,7 @@
       <c r="G121" s="31" t="s">
         <v>1286</v>
       </c>
-      <c r="H121" s="14" t="s">
+      <c r="H121" s="63" t="s">
         <v>1287</v>
       </c>
       <c r="I121" s="13" t="s">
@@ -34651,7 +34661,7 @@
       <c r="J123" s="34" t="s">
         <v>1315</v>
       </c>
-      <c r="K123" s="63" t="s">
+      <c r="K123" s="14" t="s">
         <v>1316</v>
       </c>
     </row>
@@ -35377,7 +35387,7 @@
       <c r="J145" s="4" t="s">
         <v>1529</v>
       </c>
-      <c r="K145" s="63" t="s">
+      <c r="K145" s="14" t="s">
         <v>1530</v>
       </c>
     </row>

</xml_diff>